<commit_message>
Se recortó el archivo base, a solo 2002 - 2020/02 y se aplicó la pruena de estacionalidad.
</commit_message>
<xml_diff>
--- a/outputs/resultados_estacionalidad.xlsx
+++ b/outputs/resultados_estacionalidad.xlsx
@@ -455,13 +455,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0389587757135496</v>
+        <v>0.03348431805752523</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9999993341846564</v>
+        <v>0.9999996980781836</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -481,13 +481,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7693797182775487</v>
+        <v>1.129711755685834</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6704820213011806</v>
+        <v>0.339578851153201</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -507,13 +507,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="C4" t="n">
-        <v>0.03296953335549987</v>
+        <v>0.1046006381564307</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9999997263252739</v>
+        <v>0.9998875350083889</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -533,13 +533,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="C5" t="n">
-        <v>1.21671556734702</v>
+        <v>1.238677026310312</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2763244811115435</v>
+        <v>0.2632174139134437</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -559,13 +559,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="C6" t="n">
-        <v>0.02852721646890002</v>
+        <v>0.01561397640570797</v>
       </c>
       <c r="D6" t="n">
-        <v>0.9999998738501349</v>
+        <v>0.9999999950398832</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -585,13 +585,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="C7" t="n">
-        <v>0.1986872498793383</v>
+        <v>0.1263124648951139</v>
       </c>
       <c r="D7" t="n">
-        <v>0.9975798747790234</v>
+        <v>0.9997141072260992</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -611,13 +611,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="C8" t="n">
-        <v>0.07304147968990174</v>
+        <v>0.08725656552014492</v>
       </c>
       <c r="D8" t="n">
-        <v>0.9999820837235924</v>
+        <v>0.9999548867345676</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -637,13 +637,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="C9" t="n">
-        <v>2.524254036698135</v>
+        <v>2.638197803720992</v>
       </c>
       <c r="D9" t="n">
-        <v>0.005000309598628586</v>
+        <v>0.003563164707518478</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -663,13 +663,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="C10" t="n">
-        <v>0.05391906163418454</v>
+        <v>0.07801024464060342</v>
       </c>
       <c r="D10" t="n">
-        <v>0.9999962998975589</v>
+        <v>0.9999745220166362</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -689,13 +689,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="C11" t="n">
-        <v>2.984843479929008</v>
+        <v>2.736185012107882</v>
       </c>
       <c r="D11" t="n">
-        <v>0.0009740409501628508</v>
+        <v>0.002535507330298936</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -715,13 +715,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="C12" t="n">
-        <v>0.06417323474144111</v>
+        <v>0.02262157215088239</v>
       </c>
       <c r="D12" t="n">
-        <v>0.9999908250463421</v>
+        <v>0.9999999631729491</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -741,13 +741,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="C13" t="n">
-        <v>0.2450475560704212</v>
+        <v>0.4681005308429183</v>
       </c>
       <c r="D13" t="n">
-        <v>0.9938282175235607</v>
+        <v>0.921286781752739</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>

</xml_diff>